<commit_message>
fix(income): accept INR converted columns and scan workbookPr linearly
give.do fills the converted currency and amount columns with INR on
domestic donations, so the foreign-currency guard now rejects a row
only when Donation Currency or a present Converted Currency is not INR,
ignoring case and whitespace. The synthetic fixture mirrors that.

Read the 1904 date flag with a bounded linear scan of the first
workbookPr start tag instead of a regex that was quadratic on repeated
unclosed tags.
</commit_message>
<xml_diff>
--- a/packages/e2e/fixtures/give-do/payout-sample.xlsx
+++ b/packages/e2e/fixtures/give-do/payout-sample.xlsx
@@ -266,13 +266,11 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">INR</t>
+        </is>
+      </c>
+      <c r="V2">
+        <v>1000</v>
       </c>
       <c r="W2">
         <v>25</v>
@@ -387,13 +385,11 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">INR</t>
+        </is>
+      </c>
+      <c r="V3">
+        <v>500</v>
       </c>
       <c r="W3">
         <v>12</v>

</xml_diff>